<commit_message>
Charge room cost by procedure duration
Replaces the flat operational-expense percentage with the room-hour rate
from the Hora Sala tab, prorated by how long the procedure occupies the
room. Adds a duration field, links the two tabs, and withholds the margin
verdict until clinic data exists, so a missing room cost cannot read as a
healthy margin. Clinic data now persists between sessions.

Applied to the web app, the spreadsheet, and the PDF.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Ilikia - Precificacao.xlsx
+++ b/Ilikia - Precificacao.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marti\AppData\Local\Temp\claude\C--Users-marti-OneDrive-Desktop-CLAUDE\cc5bb21a-e7ba-45a5-9ee1-3b9cb4a2d5bc\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A3ADD39-C848-49DE-8793-BD905B565102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9232EB7D-C5C0-47E5-9013-07F6F42C6BC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0E063045-8F0A-4FCF-8037-F4FEADEFF56F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{4F85614D-3B9E-4BE3-89E4-929542AFA207}"/>
   </bookViews>
   <sheets>
     <sheet name="Precificacao" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="77">
   <si>
     <t>ILIKIA · Ficha de Precificação</t>
   </si>
@@ -51,7 +51,7 @@
     <t>COMO USAR</t>
   </si>
   <si>
-    <t>Preencha apenas as células destacadas em amarelo. Todas as demais são calculadas automaticamente.</t>
+    <t>Preencha apenas as células destacadas em amarelo. Antes, preencha a aba "Hora Sala" — é de lá que vem o custo da sala.</t>
   </si>
   <si>
     <t>DADOS DO PROCEDIMENTO</t>
@@ -66,6 +66,12 @@
     <t>Valor de venda</t>
   </si>
   <si>
+    <t>Tempo do procedimento (minutos)</t>
+  </si>
+  <si>
+    <t>tempo de ocupação da sala</t>
+  </si>
+  <si>
     <t>Alíquota de imposto</t>
   </si>
   <si>
@@ -84,12 +90,6 @@
     <t>Honorário médico</t>
   </si>
   <si>
-    <t>Despesas operacionais</t>
-  </si>
-  <si>
-    <t>sobre o valor de venda</t>
-  </si>
-  <si>
     <t>INSUMOS — FICHA TÉCNICA</t>
   </si>
   <si>
@@ -108,6 +108,18 @@
     <t>TOTAL DE INSUMOS</t>
   </si>
   <si>
+    <t>CUSTO DA SALA</t>
+  </si>
+  <si>
+    <t>vem da aba "Hora Sala", proporcional ao tempo</t>
+  </si>
+  <si>
+    <t>Valor da hora sala</t>
+  </si>
+  <si>
+    <t>Custo da sala neste procedimento</t>
+  </si>
+  <si>
     <t>RESULTADO</t>
   </si>
   <si>
@@ -132,7 +144,7 @@
     <t>MARGEM DE CONTRIBUIÇÃO</t>
   </si>
   <si>
-    <t>(-) Despesas operacionais</t>
+    <t>(-) Custo da sala</t>
   </si>
   <si>
     <t>RESULTADO FINAL</t>
@@ -147,10 +159,10 @@
     <t>Verde: acima de 20%   ·   Amarelo: entre 10% e 20%   ·   Vermelho: abaixo de 10%</t>
   </si>
   <si>
-    <t>A régua de cor avalia o resultado final líquido, já descontadas as despesas operacionais.</t>
-  </si>
-  <si>
-    <t>O custo da sala não entra aqui: ele compõe as despesas operacionais e é calculado na aba "Hora Sala".</t>
+    <t>A régua de cor avalia o resultado final líquido, já descontado o custo da sala.</t>
+  </si>
+  <si>
+    <t>O custo da sala substitui a antiga despesa operacional fixa: agora ele é proporcional ao tempo que o procedimento ocupa a sala.</t>
   </si>
   <si>
     <t>ILIKIA · Cálculo da Hora Sala</t>
@@ -252,7 +264,7 @@
     <t>VALOR DA HORA SALA</t>
   </si>
   <si>
-    <t>por hora efetivamente utilizada</t>
+    <t>alimenta o custo da sala na aba Precificacao</t>
   </si>
   <si>
     <t>A hora sala custa mais que o custo de capacidade cheia porque as horas ociosas também precisam ser pagas.</t>
@@ -270,7 +282,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -321,6 +333,12 @@
       <b/>
       <sz val="12"/>
       <color rgb="FF11565E"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1E6B2E"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -462,7 +480,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -474,36 +492,39 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="3" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="6" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="13" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
     <dxf>
       <font>
         <b/>
@@ -513,6 +534,18 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFBE7E7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <color rgb="FF6E7C7D"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDED8D1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -570,13 +603,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1095375</xdr:colOff>
+      <xdr:colOff>971550</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1439018</xdr:colOff>
+      <xdr:colOff>1242168</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>330200</xdr:rowOff>
     </xdr:to>
@@ -585,7 +618,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2B6661C8-BBBE-A2C0-4C80-B0016CD9D28F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{205E86DF-8481-BF3E-95F5-AAEAB3EF8072}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -625,13 +658,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1095375</xdr:colOff>
+      <xdr:colOff>971550</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1439018</xdr:colOff>
+      <xdr:colOff>1242168</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>330200</xdr:rowOff>
     </xdr:to>
@@ -640,7 +673,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7210976F-29C5-7318-8693-C220939B86A3}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{174C5723-C67D-9A3A-D2DB-4E657F64D15E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -991,17 +1024,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CEE5F07-CE22-4785-88D7-3187CCFE6E43}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B548CBDB-FB38-41FD-98B9-C606CA4B26DB}">
   <dimension ref="A1:E60"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="38.7109375" style="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="40.6328125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="24.6328125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="38.6328125" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1010,7 +1043,7 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -1019,14 +1052,14 @@
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
     </row>
-    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>2</v>
       </c>
@@ -1035,7 +1068,7 @@
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
@@ -1044,14 +1077,14 @@
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
     </row>
-    <row r="7" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
         <v>4</v>
       </c>
@@ -1060,7 +1093,7 @@
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
@@ -1071,7 +1104,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
@@ -1082,82 +1115,82 @@
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B10" s="11">
-        <v>0.12</v>
-      </c>
-      <c r="C10" s="4"/>
+        <v>60</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>9</v>
+      </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="11">
-        <v>0.02</v>
+        <v>10</v>
+      </c>
+      <c r="B11" s="12">
+        <v>0.12</v>
       </c>
       <c r="C11" s="4"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" s="5" t="s">
         <v>11</v>
+      </c>
+      <c r="B12" s="12">
+        <v>0.02</v>
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="11">
-        <v>0.01</v>
+      <c r="B13" s="5" t="s">
+        <v>13</v>
       </c>
       <c r="C13" s="4"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" s="11">
-        <v>0.6</v>
+        <v>14</v>
+      </c>
+      <c r="B14" s="12">
+        <v>0.01</v>
       </c>
       <c r="C14" s="4"/>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15" s="11">
-        <v>0.2</v>
-      </c>
-      <c r="C15" s="4" t="s">
         <v>15</v>
       </c>
+      <c r="B15" s="12">
+        <v>0.6</v>
+      </c>
+      <c r="C15" s="4"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="4"/>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
     </row>
-    <row r="17" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A17" s="8" t="s">
         <v>16</v>
       </c>
@@ -1168,7 +1201,7 @@
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="9" t="s">
         <v>18</v>
       </c>
@@ -1179,7 +1212,7 @@
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>20</v>
       </c>
@@ -1190,74 +1223,74 @@
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="5"/>
       <c r="B20" s="10"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="5"/>
       <c r="B21" s="10"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="5"/>
       <c r="B22" s="10"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="5"/>
       <c r="B23" s="10"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="5"/>
       <c r="B24" s="10"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="5"/>
       <c r="B25" s="10"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="5"/>
       <c r="B26" s="10"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="5"/>
       <c r="B27" s="10"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="5"/>
       <c r="B28" s="10"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="13" t="s">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B29" s="14">
+      <c r="B29" s="16">
         <f>SUM(B19:B28)</f>
         <v>15</v>
       </c>
@@ -1265,14 +1298,14 @@
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
     </row>
-    <row r="31" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A31" s="8" t="s">
         <v>22</v>
       </c>
@@ -1283,267 +1316,281 @@
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B32" s="12">
-        <f>B9</f>
-        <v>500</v>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="B32" s="18">
+        <f>'Hora Sala'!$B$38</f>
+        <v>100</v>
       </c>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="21" t="s">
-        <v>24</v>
-      </c>
-      <c r="B33" s="22">
-        <f>B9*B10</f>
-        <v>60</v>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B33" s="14">
+        <f>B32*(B10/60)</f>
+        <v>100</v>
       </c>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="B34" s="22">
-        <f>B9*B11</f>
-        <v>10</v>
-      </c>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34" s="3"/>
+      <c r="B34" s="3"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="21" t="s">
+    <row r="35" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A35" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B35" s="22">
-        <f>B29</f>
-        <v>15</v>
-      </c>
-      <c r="C35" s="3"/>
+      <c r="B35" s="3"/>
+      <c r="C35" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="B36" s="22">
-        <f>B9*B14</f>
-        <v>300</v>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B36" s="13">
+        <f>B9</f>
+        <v>500</v>
       </c>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="21" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A37" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B37" s="22">
-        <f>B9*B13</f>
-        <v>5</v>
+      <c r="B37" s="26">
+        <f>B9*B11</f>
+        <v>60</v>
       </c>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="9" t="s">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A38" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="B38" s="16">
-        <f>B32-B33-B34-B35-B36-B37</f>
-        <v>110</v>
-      </c>
-      <c r="C38" s="17">
-        <f>IFERROR(B38/$B$9,0)</f>
-        <v>0.22</v>
-      </c>
+      <c r="B38" s="26">
+        <f>B9*B12</f>
+        <v>10</v>
+      </c>
+      <c r="C38" s="3"/>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A39" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="B39" s="12">
-        <f>B9*B15</f>
-        <v>100</v>
+      <c r="B39" s="26">
+        <f>B29</f>
+        <v>15</v>
       </c>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
     </row>
-    <row r="40" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A40" s="18" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A40" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="B40" s="19">
-        <f>B38-B39</f>
-        <v>10</v>
-      </c>
-      <c r="C40" s="20">
-        <f>IFERROR(B40/$B$9,0)</f>
-        <v>0.02</v>
-      </c>
+      <c r="B40" s="26">
+        <f>B9*B15</f>
+        <v>300</v>
+      </c>
+      <c r="C40" s="3"/>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="3"/>
-      <c r="B41" s="3"/>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A41" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="B41" s="26">
+        <f>B9*B14</f>
+        <v>5</v>
+      </c>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
     </row>
-    <row r="42" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A42" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B42" s="23" t="str">
-        <f>IF($B$9=0,"Informe o valor de venda para calcular",IF(C40&gt;0.2,"Margem saudável — acima da meta de 20%",IF(C40&gt;=0.1,"Margem de atenção — entre 10% e 20%","Margem crítica — abaixo de 10%")))</f>
-        <v>Margem crítica — abaixo de 10%</v>
-      </c>
-      <c r="C42" s="3"/>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A42" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B42" s="20">
+        <f>B36-B37-B38-B39-B40-B41</f>
+        <v>110</v>
+      </c>
+      <c r="C42" s="21">
+        <f>IFERROR(B42/$B$9,0)</f>
+        <v>0.22</v>
+      </c>
       <c r="D42" s="3"/>
       <c r="E42" s="3"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="3"/>
-      <c r="B43" s="3"/>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A43" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="B43" s="26">
+        <f>B33</f>
+        <v>100</v>
+      </c>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="B44" s="3"/>
-      <c r="C44" s="3"/>
+    <row r="44" spans="1:5" ht="17" x14ac:dyDescent="0.4">
+      <c r="A44" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="B44" s="23">
+        <f>B42-B43</f>
+        <v>10</v>
+      </c>
+      <c r="C44" s="24">
+        <f>IFERROR(B44/$B$9,0)</f>
+        <v>0.02</v>
+      </c>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="6" t="s">
-        <v>34</v>
-      </c>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A45" s="3"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
       <c r="E45" s="3"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B46" s="3"/>
+    <row r="46" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A46" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B46" s="27" t="str">
+        <f>IF($B$9=0,"Informe o valor de venda para calcular",IF($B$10=0,"Informe o tempo do procedimento",IF($B$32=0,"Preencha a aba Hora Sala para apurar o custo da sala",IF(C44&gt;0.2,"Margem saudável — acima da meta de 20%",IF(C44&gt;=0.1,"Margem de atenção — entre 10% e 20%","Margem crítica — abaixo de 10%")))))</f>
+        <v>Margem crítica — abaixo de 10%</v>
+      </c>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
       <c r="E46" s="3"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="6"/>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A47" s="3"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
       <c r="E47" s="3"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
       <c r="E48" s="3"/>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="3"/>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A49" s="6" t="s">
+        <v>38</v>
+      </c>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
       <c r="E49" s="3"/>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="3"/>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A50" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>
       <c r="E50" s="3"/>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="3"/>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A51" s="6"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="3"/>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A52" s="6" t="s">
+        <v>40</v>
+      </c>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
       <c r="E53" s="3"/>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
       <c r="E54" s="3"/>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
       <c r="E55" s="3"/>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
       <c r="D56" s="3"/>
       <c r="E56" s="3"/>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
       <c r="D57" s="3"/>
       <c r="E57" s="3"/>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
       <c r="D58" s="3"/>
       <c r="E58" s="3"/>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
       <c r="D59" s="3"/>
       <c r="E59" s="3"/>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
@@ -1551,20 +1598,23 @@
       <c r="E60" s="3"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C40">
-    <cfRule type="cellIs" dxfId="3" priority="1" stopIfTrue="1" operator="greaterThan">
+  <conditionalFormatting sqref="C44">
+    <cfRule type="cellIs" dxfId="4" priority="2" stopIfTrue="1" operator="greaterThan">
       <formula>0.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="2" stopIfTrue="1" operator="between">
+    <cfRule type="cellIs" dxfId="3" priority="3" stopIfTrue="1" operator="between">
       <formula>0.1</formula>
       <formula>0.2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="3" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="4" stopIfTrue="1" operator="lessThan">
       <formula>0.1</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+      <formula>$B$32=0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B12" xr:uid="{5AC279E5-2AA7-4CD8-B2E6-E7EAFDCED3C9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B13" xr:uid="{68441FC1-912C-4279-894D-A8F400255B57}">
       <formula1>"Sem antecipacao,Com antecipacao"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1574,42 +1624,42 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97D1ED72-CE67-4F74-BC1F-CA431CF06563}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A70F4CF-D349-404A-8336-660F1C8F2951}">
   <dimension ref="A1:E60"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24.7109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="38.7109375" style="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="40.6328125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="24.6328125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="38.6328125" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
     </row>
-    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>2</v>
       </c>
@@ -1618,34 +1668,34 @@
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
     </row>
-    <row r="7" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B8" s="10">
         <v>40000</v>
@@ -1654,182 +1704,182 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B9" s="24">
+        <v>46</v>
+      </c>
+      <c r="B9" s="11">
         <v>4</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B10" s="24">
+        <v>48</v>
+      </c>
+      <c r="B10" s="11">
         <v>8</v>
       </c>
       <c r="C10" s="4"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B11" s="24">
+        <v>49</v>
+      </c>
+      <c r="B11" s="11">
         <v>5</v>
       </c>
       <c r="C11" s="4"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B12" s="24">
+        <v>50</v>
+      </c>
+      <c r="B12" s="11">
         <v>4</v>
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="4"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
     </row>
-    <row r="14" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A14" s="8" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="4"/>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C15" s="4"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B16" s="25">
+        <v>54</v>
+      </c>
+      <c r="B16" s="28">
         <v>30</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B17" s="25">
+        <v>55</v>
+      </c>
+      <c r="B17" s="28">
         <v>25</v>
       </c>
       <c r="C17" s="4"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B18" s="25">
+        <v>56</v>
+      </c>
+      <c r="B18" s="28">
         <v>20</v>
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B19" s="25">
+        <v>57</v>
+      </c>
+      <c r="B19" s="28">
         <v>25</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B20" s="25"/>
+        <v>58</v>
+      </c>
+      <c r="B20" s="28"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B21" s="25"/>
+        <v>59</v>
+      </c>
+      <c r="B21" s="28"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B22" s="25"/>
+        <v>60</v>
+      </c>
+      <c r="B22" s="28"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B23" s="25"/>
+        <v>61</v>
+      </c>
+      <c r="B23" s="28"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B24" s="25"/>
+        <v>62</v>
+      </c>
+      <c r="B24" s="28"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B25" s="28"/>
+        <v>63</v>
+      </c>
+      <c r="B25" s="31"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="29" t="s">
-        <v>60</v>
-      </c>
-      <c r="B26" s="30">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="B26" s="33">
         <f>SUM(B16:B25)</f>
         <v>100</v>
       </c>
@@ -1837,11 +1887,11 @@
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="B27" s="27">
+        <v>65</v>
+      </c>
+      <c r="B27" s="30">
         <f>IFERROR(B26/B9,0)</f>
         <v>25</v>
       </c>
@@ -1849,11 +1899,11 @@
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B28" s="31" t="str">
+        <v>66</v>
+      </c>
+      <c r="B28" s="34" t="str">
         <f>IF(COUNT(B16:B25)=B9,"OK — salas preenchidas conferem","ATENÇÃO: preencha exatamente "&amp;B9&amp;" sala(s), uma por linha")</f>
         <v>OK — salas preenchidas conferem</v>
       </c>
@@ -1861,27 +1911,27 @@
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
     </row>
-    <row r="30" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A30" s="8" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B31" s="26">
+        <v>67</v>
+      </c>
+      <c r="B31" s="29">
         <f>B9*B10*B11*B12</f>
         <v>640</v>
       </c>
@@ -1889,11 +1939,11 @@
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B32" s="26">
+        <v>68</v>
+      </c>
+      <c r="B32" s="29">
         <f>B26*B12</f>
         <v>400</v>
       </c>
@@ -1901,11 +1951,11 @@
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="B33" s="26">
+        <v>69</v>
+      </c>
+      <c r="B33" s="29">
         <f>MAX(0,B31-B32)</f>
         <v>240</v>
       </c>
@@ -1913,11 +1963,11 @@
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="B34" s="15">
+        <v>70</v>
+      </c>
+      <c r="B34" s="19">
         <f>IFERROR(B32/B31,0)</f>
         <v>0.625</v>
       </c>
@@ -1925,11 +1975,11 @@
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="B35" s="12">
+        <v>71</v>
+      </c>
+      <c r="B35" s="13">
         <f>IFERROR(B8/B31,0)</f>
         <v>62.5</v>
       </c>
@@ -1937,11 +1987,11 @@
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="32" t="s">
-        <v>68</v>
-      </c>
-      <c r="B36" s="33">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36" s="35" t="s">
+        <v>72</v>
+      </c>
+      <c r="B36" s="36">
         <f>B33*B35</f>
         <v>15000</v>
       </c>
@@ -1949,179 +1999,179 @@
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
     </row>
-    <row r="38" spans="1:5" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A38" s="34" t="s">
-        <v>69</v>
-      </c>
-      <c r="B38" s="35">
+    <row r="38" spans="1:5" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A38" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="B38" s="38">
         <f>IFERROR(B8/B32,0)</f>
         <v>100</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="6" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
       <c r="E42" s="3"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="3"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
       <c r="E45" s="3"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="3"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
       <c r="E46" s="3"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="3"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
       <c r="E47" s="3"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="3"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
       <c r="E48" s="3"/>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="3"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
       <c r="E49" s="3"/>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="3"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>
       <c r="E50" s="3"/>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="3"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
       <c r="E53" s="3"/>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
       <c r="E54" s="3"/>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
       <c r="E55" s="3"/>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
       <c r="D56" s="3"/>
       <c r="E56" s="3"/>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
       <c r="D57" s="3"/>
       <c r="E57" s="3"/>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
       <c r="D58" s="3"/>
       <c r="E58" s="3"/>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
       <c r="D59" s="3"/>
       <c r="E59" s="3"/>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>

</xml_diff>